<commit_message>
Add 50 test cases
</commit_message>
<xml_diff>
--- a/IT23142978_Test cases.xlsx
+++ b/IT23142978_Test cases.xlsx
@@ -5,23 +5,23 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DELL\OneDrive\Desktop\IT23142978\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DELL\OneDrive\Desktop\IT23142978-final\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B1578A88-2959-490F-8D06-D3706C09D387}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B2EA0087-7EB0-43FC-9843-C9DBA755531B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="722" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="722" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Test cases" sheetId="3" r:id="rId1"/>
-    <sheet name="Sheet2" sheetId="5" r:id="rId2"/>
+    <sheet name="sheet1" sheetId="3" r:id="rId1"/>
+    <sheet name="Test cases" sheetId="5" r:id="rId2"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="287" uniqueCount="176">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="491" uniqueCount="316">
   <si>
     <t>TC ID</t>
   </si>
@@ -684,6 +684,426 @@
   </si>
   <si>
     <t>Pos_0024</t>
+  </si>
+  <si>
+    <t>Neg_0011</t>
+  </si>
+  <si>
+    <t>Neg_0012</t>
+  </si>
+  <si>
+    <t>Neg_0013</t>
+  </si>
+  <si>
+    <t>Neg_0014</t>
+  </si>
+  <si>
+    <t>Neg_0015</t>
+  </si>
+  <si>
+    <t>Neg_0016</t>
+  </si>
+  <si>
+    <t>Neg_0017</t>
+  </si>
+  <si>
+    <t>Neg_0018</t>
+  </si>
+  <si>
+    <t>Neg_0019</t>
+  </si>
+  <si>
+    <t>Neg_0020</t>
+  </si>
+  <si>
+    <t>Neg_0021</t>
+  </si>
+  <si>
+    <t>Neg_0022</t>
+  </si>
+  <si>
+    <t>Neg_0023</t>
+  </si>
+  <si>
+    <t>Neg_0024</t>
+  </si>
+  <si>
+    <t>Neg_0025</t>
+  </si>
+  <si>
+    <t>Neg_0026</t>
+  </si>
+  <si>
+    <t>Neg_0027</t>
+  </si>
+  <si>
+    <t>Neg_0028</t>
+  </si>
+  <si>
+    <t>Neg_0029</t>
+  </si>
+  <si>
+    <t>Neg_0030</t>
+  </si>
+  <si>
+    <t>Neg_0031</t>
+  </si>
+  <si>
+    <t>Neg_0032</t>
+  </si>
+  <si>
+    <t>Neg_0033</t>
+  </si>
+  <si>
+    <t>Neg_0034</t>
+  </si>
+  <si>
+    <t>Neg_0035</t>
+  </si>
+  <si>
+    <t>Neg_0036</t>
+  </si>
+  <si>
+    <t>Neg_0037</t>
+  </si>
+  <si>
+    <t>Neg_0038</t>
+  </si>
+  <si>
+    <t>Neg_0039</t>
+  </si>
+  <si>
+    <t>Neg_0040</t>
+  </si>
+  <si>
+    <t>Neg_0041</t>
+  </si>
+  <si>
+    <t>Neg_0042</t>
+  </si>
+  <si>
+    <t>Neg_0043</t>
+  </si>
+  <si>
+    <t>Neg_0044</t>
+  </si>
+  <si>
+    <t>Neg_0045</t>
+  </si>
+  <si>
+    <t>Neg_0046</t>
+  </si>
+  <si>
+    <t>Neg_0047</t>
+  </si>
+  <si>
+    <t>Neg_0048</t>
+  </si>
+  <si>
+    <t>Neg_0049</t>
+  </si>
+  <si>
+    <t>Neg_0050</t>
+  </si>
+  <si>
+    <t>oyala heta enawada?</t>
+  </si>
+  <si>
+    <t>ඔයාලා හෙට එනවාද?</t>
+  </si>
+  <si>
+    <t>ai meka karanne?</t>
+  </si>
+  <si>
+    <t>ඇයි මේක කරන්නේ?</t>
+  </si>
+  <si>
+    <t>mage potha aran denna</t>
+  </si>
+  <si>
+    <t>මගේ පොත අරන් දෙන්න</t>
+  </si>
+  <si>
+    <t>denma gedara yanna</t>
+  </si>
+  <si>
+    <t>දැන්ම ගෙදර යන්න</t>
+  </si>
+  <si>
+    <t>suba dawasak!</t>
+  </si>
+  <si>
+    <t>සුබ දවසක්!</t>
+  </si>
+  <si>
+    <t>obata suba pathanawa</t>
+  </si>
+  <si>
+    <t>ඔබට සුබ පතනවා</t>
+  </si>
+  <si>
+    <t>mata udaw karanna puluwanda</t>
+  </si>
+  <si>
+    <t>මට උදව් කරන්න පුළුවන්ද</t>
+  </si>
+  <si>
+    <t>karunakara meka balanna</t>
+  </si>
+  <si>
+    <t>කරුණාකර මේක බලන්න</t>
+  </si>
+  <si>
+    <t>ow mama ennam</t>
+  </si>
+  <si>
+    <t>ඔව් මම එන්නම්</t>
+  </si>
+  <si>
+    <t>na mata bari</t>
+  </si>
+  <si>
+    <t>නෑ මට බැරි</t>
+  </si>
+  <si>
+    <t>tika tika weda karamu</t>
+  </si>
+  <si>
+    <t>ටික ටික වැඩ කරමු</t>
+  </si>
+  <si>
+    <t>den den yanna one</t>
+  </si>
+  <si>
+    <t>දැන් දැන් යන්න ඕනේ</t>
+  </si>
+  <si>
+    <t>mama awa!</t>
+  </si>
+  <si>
+    <t>මම ආවා!</t>
+  </si>
+  <si>
+    <t>oyata hari da...?</t>
+  </si>
+  <si>
+    <t>ඔයාට හරිද...?</t>
+  </si>
+  <si>
+    <t>mn gedara ynwa</t>
+  </si>
+  <si>
+    <t>මං ගෙදර යනවා</t>
+  </si>
+  <si>
+    <t>oya mt call krnna</t>
+  </si>
+  <si>
+    <t>ඔයා මට call කරන්න</t>
+  </si>
+  <si>
+    <t>mama ada class yanawa</t>
+  </si>
+  <si>
+    <t>මම අද class යනවා</t>
+  </si>
+  <si>
+    <t>api party ekata yanawa</t>
+  </si>
+  <si>
+    <t>අපි party එකට යනවා</t>
+  </si>
+  <si>
+    <t>mama dan very busy inne</t>
+  </si>
+  <si>
+    <t>මම දැන් very busy ඉන්නේ</t>
+  </si>
+  <si>
+    <t>api today evening ennam</t>
+  </si>
+  <si>
+    <t>අපි today evening එන්නම්</t>
+  </si>
+  <si>
+    <t>mage email eka balanna</t>
+  </si>
+  <si>
+    <t>මගේ email එක බලන්න</t>
+  </si>
+  <si>
+    <t>wifi password eka denna</t>
+  </si>
+  <si>
+    <t>wifi password එක දෙන්න</t>
+  </si>
+  <si>
+    <t>mata Telegram message ekak danna</t>
+  </si>
+  <si>
+    <t>මට Telegram message එකක් දාන්න</t>
+  </si>
+  <si>
+    <t>api Google Meet eken katha karamu</t>
+  </si>
+  <si>
+    <t>අපි Google Meet එකෙන් කතා කරමු</t>
+  </si>
+  <si>
+    <t>CV eka ada ewanna</t>
+  </si>
+  <si>
+    <t>CV එක අද එවන්න</t>
+  </si>
+  <si>
+    <t>HR ta document eka denna</t>
+  </si>
+  <si>
+    <t>HR ට document එක දෙන්න</t>
+  </si>
+  <si>
+    <t>mata lab report eka one</t>
+  </si>
+  <si>
+    <t>මට lab report එක ඕනේ</t>
+  </si>
+  <si>
+    <t>exam hall eka hoyanna</t>
+  </si>
+  <si>
+    <t>exam hall එක හොයන්න</t>
+  </si>
+  <si>
+    <t>api Kandy walata yanawa</t>
+  </si>
+  <si>
+    <t>අපි Kandy වලට යනවා</t>
+  </si>
+  <si>
+    <t>mama Colombo wala inne</t>
+  </si>
+  <si>
+    <t>මම Colombo වල ඉන්නේ</t>
+  </si>
+  <si>
+    <t>Nimal ada awe na</t>
+  </si>
+  <si>
+    <t>නිමල් අද ආවේ නෑ</t>
+  </si>
+  <si>
+    <t>Kasuni mata katha kala</t>
+  </si>
+  <si>
+    <t>කසුනි මට කතා කළා</t>
+  </si>
+  <si>
+    <t>mata 2k denna</t>
+  </si>
+  <si>
+    <t>මට 2ක් දෙන්න</t>
+  </si>
+  <si>
+    <t>3rd lesson eka balanna</t>
+  </si>
+  <si>
+    <t>3rd lesson එක බලන්න</t>
+  </si>
+  <si>
+    <t>mata Rs. 500 one</t>
+  </si>
+  <si>
+    <t>මට Rs. 500 ඕනේ</t>
+  </si>
+  <si>
+    <t>USD 20 gewanna wenawa</t>
+  </si>
+  <si>
+    <t>USD 20 ගෙවන්න වෙනවා</t>
+  </si>
+  <si>
+    <t>api 8:15AM ennam</t>
+  </si>
+  <si>
+    <t>අපි 8:15AM එන්නම්</t>
+  </si>
+  <si>
+    <t>class eka 6.30pm iwara wenawa</t>
+  </si>
+  <si>
+    <t>class එක 6.30pm ඉවර වෙනවා</t>
+  </si>
+  <si>
+    <t>meeting eka 2026-05-10ta danna</t>
+  </si>
+  <si>
+    <t>meeting එක 2026-05-10ට දාන්න</t>
+  </si>
+  <si>
+    <t>May 20 wenakan inna</t>
+  </si>
+  <si>
+    <t>May 20 වෙනකන් ඉන්න</t>
+  </si>
+  <si>
+    <t>mama 5km duwanawa</t>
+  </si>
+  <si>
+    <t>මම 5km දුවනවා</t>
+  </si>
+  <si>
+    <t>wathura 2L denna</t>
+  </si>
+  <si>
+    <t>වතුර 2L දෙන්න</t>
+  </si>
+  <si>
+    <t>ela machan api yamu</t>
+  </si>
+  <si>
+    <t>එළ මචං අපි යමු</t>
+  </si>
+  <si>
+    <t>patta wadak bn</t>
+  </si>
+  <si>
+    <t>පට්ට වැඩක් බං</t>
+  </si>
+  <si>
+    <t>me link eka open karanna: https://abc.lk</t>
+  </si>
+  <si>
+    <t>මේ link එක open කරන්න: https://abc.lk</t>
+  </si>
+  <si>
+    <t>mage email eka: nimal22@gmail.com</t>
+  </si>
+  <si>
+    <t>මගේ email එක: nimal22@gmail.com</t>
+  </si>
+  <si>
+    <t>mama dan yanawa 😂</t>
+  </si>
+  <si>
+    <t>මම දැන් යනවා 😂</t>
+  </si>
+  <si>
+    <t>eya godak hithuwakara kenek ❤️</t>
+  </si>
+  <si>
+    <t>එයා ගොඩක් හිතුවක්කාර කෙනෙක් ❤️</t>
+  </si>
+  <si>
+    <t>ane mata poddak help karanna</t>
+  </si>
+  <si>
+    <t>අනේ මට පොඩ්ඩක් help කරන්න</t>
+  </si>
+  <si>
+    <t>uba den online innawada?</t>
+  </si>
+  <si>
+    <t>උඹ දැන් online ඉන්නවාද?</t>
   </si>
 </sst>
 </file>
@@ -719,7 +1139,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -730,6 +1150,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1620,7 +2043,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="24" spans="1:8" ht="86.4" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:8" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A24" s="2" t="s">
         <v>174</v>
       </c>
@@ -1963,9 +2386,788 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E3DCF8EC-25D1-4BEE-B426-FD8D0F98085D}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:H51"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <sheetData/>
+  <cols>
+    <col min="1" max="1" width="11.109375" customWidth="1"/>
+    <col min="2" max="2" width="20.88671875" customWidth="1"/>
+    <col min="3" max="3" width="37.5546875" customWidth="1"/>
+    <col min="4" max="4" width="41" customWidth="1"/>
+    <col min="5" max="5" width="28" customWidth="1"/>
+    <col min="6" max="6" width="23.5546875" customWidth="1"/>
+    <col min="7" max="7" width="28.44140625" customWidth="1"/>
+    <col min="8" max="8" width="23" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="4"/>
+      <c r="F1" s="4"/>
+      <c r="G1" s="4"/>
+      <c r="H1" s="4"/>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A2" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="C2" s="6" t="s">
+        <v>216</v>
+      </c>
+      <c r="D2" s="6" t="s">
+        <v>217</v>
+      </c>
+      <c r="E2" s="6"/>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="C3" s="6" t="s">
+        <v>218</v>
+      </c>
+      <c r="D3" s="6" t="s">
+        <v>219</v>
+      </c>
+      <c r="E3" s="6"/>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A4" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C4" s="6" t="s">
+        <v>220</v>
+      </c>
+      <c r="D4" s="6" t="s">
+        <v>221</v>
+      </c>
+      <c r="E4" s="6"/>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A5" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C5" s="6" t="s">
+        <v>222</v>
+      </c>
+      <c r="D5" s="6" t="s">
+        <v>223</v>
+      </c>
+      <c r="E5" s="6"/>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A6" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="C6" s="6" t="s">
+        <v>224</v>
+      </c>
+      <c r="D6" s="6" t="s">
+        <v>225</v>
+      </c>
+      <c r="E6" s="6"/>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A7" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="B7" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C7" s="6" t="s">
+        <v>226</v>
+      </c>
+      <c r="D7" s="6" t="s">
+        <v>227</v>
+      </c>
+      <c r="E7" s="6"/>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A8" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="B8" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C8" s="6" t="s">
+        <v>228</v>
+      </c>
+      <c r="D8" s="6" t="s">
+        <v>229</v>
+      </c>
+      <c r="E8" s="6"/>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A9" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="B9" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C9" s="6" t="s">
+        <v>230</v>
+      </c>
+      <c r="D9" s="6" t="s">
+        <v>231</v>
+      </c>
+      <c r="E9" s="6"/>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A10" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B10" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="C10" s="6" t="s">
+        <v>232</v>
+      </c>
+      <c r="D10" s="6" t="s">
+        <v>233</v>
+      </c>
+      <c r="E10" s="6"/>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A11" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="B11" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="C11" s="6" t="s">
+        <v>234</v>
+      </c>
+      <c r="D11" s="6" t="s">
+        <v>235</v>
+      </c>
+      <c r="E11" s="6"/>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A12" s="4" t="s">
+        <v>176</v>
+      </c>
+      <c r="B12" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C12" s="6" t="s">
+        <v>236</v>
+      </c>
+      <c r="D12" s="6" t="s">
+        <v>237</v>
+      </c>
+      <c r="E12" s="6"/>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A13" s="4" t="s">
+        <v>177</v>
+      </c>
+      <c r="B13" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C13" s="6" t="s">
+        <v>238</v>
+      </c>
+      <c r="D13" s="6" t="s">
+        <v>239</v>
+      </c>
+      <c r="E13" s="6"/>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A14" s="4" t="s">
+        <v>178</v>
+      </c>
+      <c r="B14" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="C14" s="6" t="s">
+        <v>240</v>
+      </c>
+      <c r="D14" s="6" t="s">
+        <v>241</v>
+      </c>
+      <c r="E14" s="6"/>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A15" s="4" t="s">
+        <v>179</v>
+      </c>
+      <c r="B15" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C15" s="6" t="s">
+        <v>242</v>
+      </c>
+      <c r="D15" s="6" t="s">
+        <v>243</v>
+      </c>
+      <c r="E15" s="6"/>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A16" s="4" t="s">
+        <v>180</v>
+      </c>
+      <c r="B16" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C16" s="6" t="s">
+        <v>244</v>
+      </c>
+      <c r="D16" s="6" t="s">
+        <v>245</v>
+      </c>
+      <c r="E16" s="6"/>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A17" s="4" t="s">
+        <v>181</v>
+      </c>
+      <c r="B17" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C17" s="6" t="s">
+        <v>246</v>
+      </c>
+      <c r="D17" s="6" t="s">
+        <v>247</v>
+      </c>
+      <c r="E17" s="6"/>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A18" s="4" t="s">
+        <v>182</v>
+      </c>
+      <c r="B18" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C18" s="6" t="s">
+        <v>248</v>
+      </c>
+      <c r="D18" s="6" t="s">
+        <v>249</v>
+      </c>
+      <c r="E18" s="6"/>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A19" s="4" t="s">
+        <v>183</v>
+      </c>
+      <c r="B19" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C19" s="6" t="s">
+        <v>250</v>
+      </c>
+      <c r="D19" s="6" t="s">
+        <v>251</v>
+      </c>
+      <c r="E19" s="6"/>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A20" s="4" t="s">
+        <v>184</v>
+      </c>
+      <c r="B20" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C20" s="6" t="s">
+        <v>252</v>
+      </c>
+      <c r="D20" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="E20" s="6"/>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A21" s="4" t="s">
+        <v>185</v>
+      </c>
+      <c r="B21" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C21" s="6" t="s">
+        <v>254</v>
+      </c>
+      <c r="D21" s="6" t="s">
+        <v>255</v>
+      </c>
+      <c r="E21" s="6"/>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A22" s="4" t="s">
+        <v>186</v>
+      </c>
+      <c r="B22" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C22" s="6" t="s">
+        <v>256</v>
+      </c>
+      <c r="D22" s="6" t="s">
+        <v>257</v>
+      </c>
+      <c r="E22" s="6"/>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A23" s="4" t="s">
+        <v>187</v>
+      </c>
+      <c r="B23" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C23" s="6" t="s">
+        <v>258</v>
+      </c>
+      <c r="D23" s="6" t="s">
+        <v>259</v>
+      </c>
+      <c r="E23" s="6"/>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A24" s="4" t="s">
+        <v>188</v>
+      </c>
+      <c r="B24" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C24" s="6" t="s">
+        <v>260</v>
+      </c>
+      <c r="D24" s="6" t="s">
+        <v>261</v>
+      </c>
+      <c r="E24" s="6"/>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A25" s="4" t="s">
+        <v>189</v>
+      </c>
+      <c r="B25" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C25" s="6" t="s">
+        <v>262</v>
+      </c>
+      <c r="D25" s="6" t="s">
+        <v>263</v>
+      </c>
+      <c r="E25" s="6"/>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A26" s="4" t="s">
+        <v>190</v>
+      </c>
+      <c r="B26" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C26" s="6" t="s">
+        <v>264</v>
+      </c>
+      <c r="D26" s="6" t="s">
+        <v>265</v>
+      </c>
+      <c r="E26" s="6"/>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A27" s="4" t="s">
+        <v>191</v>
+      </c>
+      <c r="B27" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C27" s="6" t="s">
+        <v>266</v>
+      </c>
+      <c r="D27" s="6" t="s">
+        <v>267</v>
+      </c>
+      <c r="E27" s="6"/>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A28" s="4" t="s">
+        <v>192</v>
+      </c>
+      <c r="B28" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C28" s="6" t="s">
+        <v>268</v>
+      </c>
+      <c r="D28" s="6" t="s">
+        <v>269</v>
+      </c>
+      <c r="E28" s="6"/>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A29" s="4" t="s">
+        <v>193</v>
+      </c>
+      <c r="B29" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C29" s="6" t="s">
+        <v>270</v>
+      </c>
+      <c r="D29" s="6" t="s">
+        <v>271</v>
+      </c>
+      <c r="E29" s="6"/>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A30" s="4" t="s">
+        <v>194</v>
+      </c>
+      <c r="B30" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C30" s="6" t="s">
+        <v>272</v>
+      </c>
+      <c r="D30" s="6" t="s">
+        <v>273</v>
+      </c>
+      <c r="E30" s="6"/>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A31" s="4" t="s">
+        <v>195</v>
+      </c>
+      <c r="B31" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C31" s="6" t="s">
+        <v>274</v>
+      </c>
+      <c r="D31" s="6" t="s">
+        <v>275</v>
+      </c>
+      <c r="E31" s="6"/>
+    </row>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A32" s="4" t="s">
+        <v>196</v>
+      </c>
+      <c r="B32" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C32" s="6" t="s">
+        <v>276</v>
+      </c>
+      <c r="D32" s="6" t="s">
+        <v>277</v>
+      </c>
+      <c r="E32" s="6"/>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A33" s="4" t="s">
+        <v>197</v>
+      </c>
+      <c r="B33" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C33" s="6" t="s">
+        <v>278</v>
+      </c>
+      <c r="D33" s="6" t="s">
+        <v>279</v>
+      </c>
+      <c r="E33" s="6"/>
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A34" s="4" t="s">
+        <v>198</v>
+      </c>
+      <c r="B34" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C34" s="6" t="s">
+        <v>280</v>
+      </c>
+      <c r="D34" s="6" t="s">
+        <v>281</v>
+      </c>
+      <c r="E34" s="6"/>
+    </row>
+    <row r="35" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A35" s="4" t="s">
+        <v>199</v>
+      </c>
+      <c r="B35" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C35" s="6" t="s">
+        <v>282</v>
+      </c>
+      <c r="D35" s="6" t="s">
+        <v>283</v>
+      </c>
+      <c r="E35" s="6"/>
+    </row>
+    <row r="36" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A36" s="4" t="s">
+        <v>200</v>
+      </c>
+      <c r="B36" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C36" s="6" t="s">
+        <v>284</v>
+      </c>
+      <c r="D36" s="6" t="s">
+        <v>285</v>
+      </c>
+      <c r="E36" s="6"/>
+    </row>
+    <row r="37" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A37" s="4" t="s">
+        <v>201</v>
+      </c>
+      <c r="B37" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C37" s="6" t="s">
+        <v>286</v>
+      </c>
+      <c r="D37" s="6" t="s">
+        <v>287</v>
+      </c>
+      <c r="E37" s="6"/>
+    </row>
+    <row r="38" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A38" s="4" t="s">
+        <v>202</v>
+      </c>
+      <c r="B38" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C38" s="6" t="s">
+        <v>288</v>
+      </c>
+      <c r="D38" s="6" t="s">
+        <v>289</v>
+      </c>
+      <c r="E38" s="6"/>
+    </row>
+    <row r="39" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A39" s="4" t="s">
+        <v>203</v>
+      </c>
+      <c r="B39" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C39" s="6" t="s">
+        <v>290</v>
+      </c>
+      <c r="D39" s="6" t="s">
+        <v>291</v>
+      </c>
+      <c r="E39" s="6"/>
+    </row>
+    <row r="40" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A40" s="4" t="s">
+        <v>204</v>
+      </c>
+      <c r="B40" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C40" s="6" t="s">
+        <v>292</v>
+      </c>
+      <c r="D40" s="6" t="s">
+        <v>293</v>
+      </c>
+      <c r="E40" s="6"/>
+    </row>
+    <row r="41" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A41" s="4" t="s">
+        <v>205</v>
+      </c>
+      <c r="B41" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C41" s="6" t="s">
+        <v>294</v>
+      </c>
+      <c r="D41" s="6" t="s">
+        <v>295</v>
+      </c>
+      <c r="E41" s="6"/>
+    </row>
+    <row r="42" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A42" s="4" t="s">
+        <v>206</v>
+      </c>
+      <c r="B42" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C42" s="6" t="s">
+        <v>296</v>
+      </c>
+      <c r="D42" s="6" t="s">
+        <v>297</v>
+      </c>
+      <c r="E42" s="6"/>
+    </row>
+    <row r="43" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A43" s="4" t="s">
+        <v>207</v>
+      </c>
+      <c r="B43" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C43" s="6" t="s">
+        <v>298</v>
+      </c>
+      <c r="D43" s="6" t="s">
+        <v>299</v>
+      </c>
+      <c r="E43" s="6"/>
+    </row>
+    <row r="44" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A44" s="4" t="s">
+        <v>208</v>
+      </c>
+      <c r="B44" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C44" s="6" t="s">
+        <v>300</v>
+      </c>
+      <c r="D44" s="6" t="s">
+        <v>301</v>
+      </c>
+      <c r="E44" s="6"/>
+    </row>
+    <row r="45" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A45" s="4" t="s">
+        <v>209</v>
+      </c>
+      <c r="B45" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C45" s="6" t="s">
+        <v>302</v>
+      </c>
+      <c r="D45" s="6" t="s">
+        <v>303</v>
+      </c>
+      <c r="E45" s="6"/>
+    </row>
+    <row r="46" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A46" s="4" t="s">
+        <v>210</v>
+      </c>
+      <c r="B46" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C46" s="6" t="s">
+        <v>304</v>
+      </c>
+      <c r="D46" s="6" t="s">
+        <v>305</v>
+      </c>
+      <c r="E46" s="6"/>
+    </row>
+    <row r="47" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A47" s="4" t="s">
+        <v>211</v>
+      </c>
+      <c r="B47" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C47" s="6" t="s">
+        <v>306</v>
+      </c>
+      <c r="D47" s="6" t="s">
+        <v>307</v>
+      </c>
+      <c r="E47" s="6"/>
+    </row>
+    <row r="48" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A48" s="4" t="s">
+        <v>212</v>
+      </c>
+      <c r="B48" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C48" s="6" t="s">
+        <v>308</v>
+      </c>
+      <c r="D48" s="6" t="s">
+        <v>309</v>
+      </c>
+      <c r="E48" s="6"/>
+    </row>
+    <row r="49" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A49" s="4" t="s">
+        <v>213</v>
+      </c>
+      <c r="B49" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C49" s="6" t="s">
+        <v>310</v>
+      </c>
+      <c r="D49" s="6" t="s">
+        <v>311</v>
+      </c>
+      <c r="E49" s="6"/>
+    </row>
+    <row r="50" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A50" s="4" t="s">
+        <v>214</v>
+      </c>
+      <c r="B50" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C50" s="6" t="s">
+        <v>312</v>
+      </c>
+      <c r="D50" s="6" t="s">
+        <v>313</v>
+      </c>
+      <c r="E50" s="6"/>
+    </row>
+    <row r="51" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A51" s="4" t="s">
+        <v>215</v>
+      </c>
+      <c r="B51" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C51" s="6" t="s">
+        <v>314</v>
+      </c>
+      <c r="D51" s="6" t="s">
+        <v>315</v>
+      </c>
+      <c r="E51" s="6"/>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Complete 50 test cases with input types and rationale
</commit_message>
<xml_diff>
--- a/IT23142978_Test cases.xlsx
+++ b/IT23142978_Test cases.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DELL\OneDrive\Desktop\IT23142978\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D4DE5DE2-28B0-4DA1-B5F2-9ED6B84ABFD9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{79A1924F-B591-4683-9E12-84EE85E85103}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="722" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1178,7 +1178,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="22.8" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>6</v>
       </c>
@@ -1204,7 +1204,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="3" spans="1:8" ht="34.200000000000003" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:8" ht="22.8" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>9</v>
       </c>
@@ -1230,7 +1230,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="22.8" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
         <v>10</v>
       </c>
@@ -1542,7 +1542,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="16" spans="1:8" ht="34.200000000000003" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:8" ht="22.8" x14ac:dyDescent="0.3">
       <c r="A16" s="2" t="s">
         <v>23</v>
       </c>

</xml_diff>